<commit_message>
Fix logistics master costs and store grouping
</commit_message>
<xml_diff>
--- a/유월의보리_product_master.xlsx
+++ b/유월의보리_product_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\STAND UP\Desktop\HQ\본사 물류마감 자료\26_05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C10FE60-65DA-4456-9EE7-874865A9F986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E99D747-4CF7-4D52-A7BF-9A7B4FEE266E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -606,10 +606,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="176" formatCode="0.0%"/>
-    <numFmt numFmtId="180" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -700,6 +700,11 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -784,14 +789,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="180" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -807,16 +812,6 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -847,9 +842,23 @@
     <xf numFmtId="49" fontId="9" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="15" fillId="7" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -861,101 +870,9 @@
     <cellStyle name="표준 2 2" xfId="6" xr:uid="{2855F415-4440-4082-81F9-DE5C7481323B}"/>
     <cellStyle name="표준 3" xfId="3" xr:uid="{5BFFED80-3383-433D-A609-A987DBFBC66D}"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="15">
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <sz val="12"/>
-        <color theme="0"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Carlito"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill>
           <fgColor indexed="64"/>
@@ -980,6 +897,20 @@
           <color indexed="64"/>
         </horizontal>
       </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -1182,19 +1113,105 @@
           <bgColor theme="0"/>
         </patternFill>
       </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFEE2E2"/>
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Carlito"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <sz val="12"/>
+        <color theme="0"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="SlicerStyleLight1 Dark" pivot="0" table="0" count="2" xr9:uid="{51F6AAFE-A6A2-4D1B-994A-EE3C093D1FD8}">
-      <tableStyleElement type="wholeTable" dxfId="1"/>
-      <tableStyleElement type="headerRow" dxfId="0"/>
+      <tableStyleElement type="wholeTable" dxfId="14"/>
+      <tableStyleElement type="headerRow" dxfId="13"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1209,20 +1226,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProductMasterTable" displayName="ProductMasterTable" ref="A1:H45" headerRowDxfId="3" dataDxfId="12" totalsRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProductMasterTable" displayName="ProductMasterTable" ref="A1:H45" headerRowDxfId="12" dataDxfId="11" totalsRowDxfId="10">
   <autoFilter ref="A1:H45" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H35">
     <sortCondition ref="B1:B35"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="사용여부" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="품목코드" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="품목명(규격)" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="구분" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="공급단가(ERP)" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="제조원가(입력)" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="팩/단위" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="비고" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="사용여부" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="품목코드" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="품목명(규격)" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="구분" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="공급단가(ERP)" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="제조원가(입력)" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="팩/단위" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="비고" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1398,1084 +1415,1137 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="9" style="18" customWidth="1"/>
-    <col min="2" max="2" width="13" style="18" customWidth="1"/>
-    <col min="3" max="3" width="39.09765625" style="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12" style="18" customWidth="1"/>
-    <col min="5" max="5" width="14" style="18" customWidth="1"/>
-    <col min="6" max="6" width="15" style="18" customWidth="1"/>
-    <col min="7" max="7" width="12" style="18" customWidth="1"/>
-    <col min="8" max="8" width="24" style="18" customWidth="1"/>
-    <col min="9" max="16384" width="8.796875" style="11"/>
+    <col min="1" max="1" width="9" style="14" customWidth="1"/>
+    <col min="2" max="2" width="13" style="14" customWidth="1"/>
+    <col min="3" max="3" width="39.09765625" style="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" style="14" customWidth="1"/>
+    <col min="5" max="5" width="14" style="14" customWidth="1"/>
+    <col min="6" max="6" width="15" style="14" customWidth="1"/>
+    <col min="7" max="7" width="12" style="14" customWidth="1"/>
+    <col min="8" max="8" width="24" style="14" customWidth="1"/>
+    <col min="9" max="16384" width="8.796875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="12" customFormat="1">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:10" s="8" customFormat="1">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="9" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="14" t="s">
+      <c r="J1" s="23"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="16">
+      <c r="E2" s="12">
         <v>23000</v>
       </c>
-      <c r="F2" s="16">
+      <c r="F2" s="12">
         <v>23000</v>
       </c>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-    </row>
-    <row r="3" spans="1:8" ht="17.399999999999999">
-      <c r="A3" s="14" t="s">
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="J2" s="23"/>
+    </row>
+    <row r="3" spans="1:10" ht="17.399999999999999">
+      <c r="A3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="12">
         <v>28000</v>
       </c>
-      <c r="F3" s="16">
+      <c r="F3" s="12">
         <v>28000</v>
       </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="14" t="s">
+      <c r="J3" s="23"/>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="19">
+      <c r="E4" s="15">
         <v>41700</v>
       </c>
-      <c r="F4" s="16">
-        <v>80724</v>
-      </c>
-      <c r="G4" s="23" t="s">
+      <c r="F4" s="12">
+        <v>20181</v>
+      </c>
+      <c r="G4" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H4" s="14"/>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="14" t="s">
+      <c r="H4" s="10"/>
+      <c r="J4" s="23"/>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="19">
+      <c r="E5" s="15">
         <v>36000</v>
       </c>
-      <c r="F5" s="16">
-        <v>79892</v>
-      </c>
-      <c r="G5" s="23" t="s">
+      <c r="F5" s="12">
+        <v>19973</v>
+      </c>
+      <c r="G5" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H5" s="14"/>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="14" t="s">
+      <c r="H5" s="10"/>
+      <c r="J5" s="23"/>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="15">
         <v>26800</v>
       </c>
-      <c r="F6" s="16">
-        <v>73780</v>
-      </c>
-      <c r="G6" s="23" t="s">
+      <c r="F6" s="12">
+        <v>18445</v>
+      </c>
+      <c r="G6" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H6" s="14"/>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="14" t="s">
+      <c r="H6" s="10"/>
+      <c r="J6" s="23"/>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="15">
         <v>18000</v>
       </c>
-      <c r="F7" s="16">
-        <v>26812</v>
-      </c>
-      <c r="G7" s="23" t="s">
+      <c r="F7" s="12">
+        <v>6703</v>
+      </c>
+      <c r="G7" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H7" s="14"/>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="14" t="s">
+      <c r="H7" s="10"/>
+      <c r="J7" s="23"/>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="15">
         <v>29000</v>
       </c>
-      <c r="F8" s="16">
-        <v>62180</v>
-      </c>
-      <c r="G8" s="23" t="s">
+      <c r="F8" s="12">
+        <v>15545</v>
+      </c>
+      <c r="G8" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H8" s="14"/>
-    </row>
-    <row r="9" spans="1:8" ht="17.399999999999999" customHeight="1">
-      <c r="A9" s="14" t="s">
+      <c r="H8" s="10"/>
+      <c r="J8" s="23"/>
+    </row>
+    <row r="9" spans="1:10" ht="17.399999999999999" customHeight="1">
+      <c r="A9" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="15">
         <v>29000</v>
       </c>
-      <c r="F9" s="16">
-        <v>52960</v>
-      </c>
-      <c r="G9" s="23" t="s">
+      <c r="F9" s="12">
+        <v>13240</v>
+      </c>
+      <c r="G9" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H9" s="14"/>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="14" t="s">
+      <c r="H9" s="10"/>
+      <c r="J9" s="23"/>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="C10" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="D10" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="15">
         <v>85756</v>
       </c>
-      <c r="F10" s="16">
+      <c r="F10" s="12">
         <v>34600</v>
       </c>
-      <c r="G10" s="23" t="s">
+      <c r="G10" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H10" s="14"/>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="14" t="s">
+      <c r="H10" s="10"/>
+      <c r="J10" s="23"/>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="C11" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="15">
         <v>20835</v>
       </c>
-      <c r="F11" s="16">
-        <v>31240</v>
-      </c>
-      <c r="G11" s="23" t="s">
+      <c r="F11" s="12">
+        <v>7810</v>
+      </c>
+      <c r="G11" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H11" s="14"/>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="14" t="s">
+      <c r="H11" s="10"/>
+      <c r="J11" s="24"/>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="19">
+      <c r="E12" s="15">
         <v>56200</v>
       </c>
-      <c r="F12" s="16">
-        <v>104332</v>
-      </c>
-      <c r="G12" s="23" t="s">
+      <c r="F12" s="12">
+        <v>26083</v>
+      </c>
+      <c r="G12" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H12" s="14"/>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" s="14" t="s">
+      <c r="H12" s="10"/>
+      <c r="J12" s="24"/>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="C13" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="19">
+      <c r="E13" s="15">
         <v>36300</v>
       </c>
-      <c r="F13" s="16">
-        <v>60128</v>
-      </c>
-      <c r="G13" s="23" t="s">
+      <c r="F13" s="12">
+        <v>15032</v>
+      </c>
+      <c r="G13" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H13" s="14"/>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" s="14" t="s">
+      <c r="H13" s="10"/>
+      <c r="J13" s="24"/>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="C14" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="19">
+      <c r="E14" s="15">
         <v>43200</v>
       </c>
-      <c r="F14" s="20">
-        <v>34500</v>
-      </c>
-      <c r="G14" s="23" t="s">
+      <c r="F14" s="16">
+        <v>17850</v>
+      </c>
+      <c r="G14" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H14" s="14"/>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" s="14" t="s">
+      <c r="H14" s="10"/>
+      <c r="J14" s="24"/>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="22" t="s">
+      <c r="C15" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="D15" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E15" s="19">
+      <c r="E15" s="15">
         <v>31900</v>
       </c>
-      <c r="F15" s="20">
-        <v>7303</v>
-      </c>
-      <c r="G15" s="23" t="s">
+      <c r="F15" s="16">
+        <v>7300</v>
+      </c>
+      <c r="G15" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H15" s="14"/>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" s="14" t="s">
+      <c r="H15" s="10"/>
+      <c r="J15" s="24"/>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="D16" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E16" s="19">
+      <c r="E16" s="15">
         <v>27700</v>
       </c>
-      <c r="F16" s="20">
+      <c r="F16" s="16">
         <v>4125</v>
       </c>
-      <c r="G16" s="23" t="s">
+      <c r="G16" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="H16" s="14"/>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" s="14" t="s">
+      <c r="H16" s="10"/>
+      <c r="J16" s="24"/>
+    </row>
+    <row r="17" spans="1:10">
+      <c r="A17" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="D17" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E17" s="19">
+      <c r="E17" s="15">
         <v>89200</v>
       </c>
-      <c r="F17" s="20">
-        <v>15703</v>
-      </c>
-      <c r="G17" s="23" t="s">
+      <c r="F17" s="16">
+        <v>11670</v>
+      </c>
+      <c r="G17" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="H17" s="14"/>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" s="14" t="s">
+      <c r="H17" s="10"/>
+      <c r="J17" s="24"/>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="A18" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E18" s="19">
+      <c r="E18" s="15">
         <v>22000</v>
       </c>
-      <c r="F18" s="20">
-        <v>36664.800000000003</v>
-      </c>
-      <c r="G18" s="23" t="s">
+      <c r="F18" s="16">
+        <v>9180</v>
+      </c>
+      <c r="G18" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="H18" s="14"/>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" s="14" t="s">
+      <c r="H18" s="10"/>
+      <c r="J18" s="24"/>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="19">
+      <c r="E19" s="15">
         <v>20000</v>
       </c>
-      <c r="F19" s="20">
-        <v>41767.199999999997</v>
-      </c>
-      <c r="G19" s="23" t="s">
+      <c r="F19" s="16">
+        <v>10350</v>
+      </c>
+      <c r="G19" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="H19" s="14"/>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20" s="14" t="s">
+      <c r="H19" s="10"/>
+      <c r="J19" s="24"/>
+    </row>
+    <row r="20" spans="1:10">
+      <c r="A20" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="19">
+      <c r="E20" s="15">
         <v>13500</v>
       </c>
-      <c r="F20" s="20">
-        <v>27000</v>
-      </c>
-      <c r="G20" s="23" t="s">
+      <c r="F20" s="16">
+        <v>7000</v>
+      </c>
+      <c r="G20" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="H20" s="14"/>
-    </row>
-    <row r="21" spans="1:8">
-      <c r="A21" s="14" t="s">
+      <c r="H20" s="10"/>
+      <c r="J20" s="24"/>
+    </row>
+    <row r="21" spans="1:10">
+      <c r="A21" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="D21" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E21" s="19">
+      <c r="E21" s="15">
         <v>70000</v>
       </c>
-      <c r="F21" s="20">
-        <v>72424</v>
-      </c>
-      <c r="G21" s="23" t="s">
+      <c r="F21" s="16">
+        <v>18106</v>
+      </c>
+      <c r="G21" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="H21" s="14"/>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" s="14" t="s">
+      <c r="H21" s="10"/>
+      <c r="J21" s="24"/>
+    </row>
+    <row r="22" spans="1:10">
+      <c r="A22" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C22" s="22" t="s">
+      <c r="C22" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="D22" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="15">
         <v>22400</v>
       </c>
-      <c r="F22" s="20">
-        <v>12450</v>
-      </c>
-      <c r="G22" s="23" t="s">
+      <c r="F22" s="16">
+        <v>3328</v>
+      </c>
+      <c r="G22" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="H22" s="14"/>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23" s="14" t="s">
+      <c r="H22" s="10"/>
+      <c r="J22" s="24"/>
+    </row>
+    <row r="23" spans="1:10">
+      <c r="A23" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B23" s="14" t="s">
+      <c r="B23" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C23" s="22" t="s">
+      <c r="C23" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="D23" s="14" t="s">
+      <c r="D23" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="15">
         <v>24000</v>
       </c>
-      <c r="F23" s="20">
-        <v>21990</v>
-      </c>
-      <c r="G23" s="23" t="s">
+      <c r="F23" s="16">
+        <v>20435</v>
+      </c>
+      <c r="G23" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H23" s="14"/>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" s="14" t="s">
+      <c r="H23" s="10"/>
+      <c r="J23" s="24"/>
+    </row>
+    <row r="24" spans="1:10">
+      <c r="A24" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="14" t="s">
+      <c r="B24" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="C24" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="D24" s="14" t="s">
+      <c r="D24" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="15">
         <v>78000</v>
       </c>
-      <c r="F24" s="20">
+      <c r="F24" s="16">
         <v>72000</v>
       </c>
-      <c r="G24" s="23" t="s">
+      <c r="G24" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="H24" s="14"/>
-    </row>
-    <row r="25" spans="1:8">
-      <c r="A25" s="14" t="s">
+      <c r="H24" s="10"/>
+      <c r="J24" s="24"/>
+    </row>
+    <row r="25" spans="1:10">
+      <c r="A25" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B25" s="14" t="s">
+      <c r="B25" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="22" t="s">
+      <c r="C25" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="D25" s="14" t="s">
+      <c r="D25" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E25" s="19">
+      <c r="E25" s="15">
         <v>22000</v>
       </c>
-      <c r="F25" s="20">
-        <v>43044</v>
-      </c>
-      <c r="G25" s="23" t="s">
+      <c r="F25" s="16">
+        <v>10761</v>
+      </c>
+      <c r="G25" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="H25" s="14"/>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" s="14" t="s">
+      <c r="H25" s="10"/>
+      <c r="J25" s="24"/>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="C26" s="18" t="s">
         <v>128</v>
       </c>
-      <c r="D26" s="14" t="s">
+      <c r="D26" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E26" s="19">
+      <c r="E26" s="15">
         <v>22000</v>
       </c>
-      <c r="F26" s="20">
-        <v>39880</v>
-      </c>
-      <c r="G26" s="23" t="s">
+      <c r="F26" s="16">
+        <v>9967</v>
+      </c>
+      <c r="G26" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="H26" s="14"/>
-    </row>
-    <row r="27" spans="1:8">
-      <c r="A27" s="14" t="s">
+      <c r="H26" s="10"/>
+      <c r="J26" s="24"/>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B27" s="14" t="s">
+      <c r="B27" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="C27" s="22" t="s">
+      <c r="C27" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="D27" s="14" t="s">
+      <c r="D27" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E27" s="19">
+      <c r="E27" s="15">
         <v>43200</v>
       </c>
-      <c r="F27" s="20">
-        <v>48214</v>
-      </c>
-      <c r="G27" s="23" t="s">
+      <c r="F27" s="16">
+        <v>24107</v>
+      </c>
+      <c r="G27" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="H27" s="14"/>
-    </row>
-    <row r="28" spans="1:8" ht="17.399999999999999" customHeight="1">
-      <c r="A28" s="14" t="s">
+      <c r="H27" s="10"/>
+      <c r="J27" s="24"/>
+    </row>
+    <row r="28" spans="1:10" ht="17.399999999999999" customHeight="1">
+      <c r="A28" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B28" s="14" t="s">
+      <c r="B28" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="D28" s="14" t="s">
+      <c r="D28" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E28" s="19">
+      <c r="E28" s="15">
         <v>20150</v>
       </c>
-      <c r="F28" s="20">
+      <c r="F28" s="16">
         <v>18150</v>
       </c>
-      <c r="G28" s="23" t="s">
+      <c r="G28" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="H28" s="14"/>
-    </row>
-    <row r="29" spans="1:8">
-      <c r="A29" s="14" t="s">
+      <c r="H28" s="10"/>
+      <c r="J28" s="25"/>
+    </row>
+    <row r="29" spans="1:10">
+      <c r="A29" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B29" s="14" t="s">
+      <c r="B29" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C29" s="22" t="s">
+      <c r="C29" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="D29" s="14" t="s">
+      <c r="D29" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E29" s="19">
+      <c r="E29" s="15">
         <v>126000</v>
       </c>
-      <c r="F29" s="20">
+      <c r="F29" s="16">
         <v>120000</v>
       </c>
-      <c r="G29" s="23" t="s">
+      <c r="G29" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="H29" s="14"/>
-    </row>
-    <row r="30" spans="1:8">
-      <c r="A30" s="14" t="s">
+      <c r="H29" s="10"/>
+      <c r="J29" s="24"/>
+    </row>
+    <row r="30" spans="1:10">
+      <c r="A30" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="B30" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C30" s="22" t="s">
+      <c r="C30" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="D30" s="14" t="s">
+      <c r="D30" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E30" s="19">
+      <c r="E30" s="15">
         <v>40200</v>
       </c>
-      <c r="F30" s="20">
+      <c r="F30" s="16">
         <v>35200</v>
       </c>
-      <c r="G30" s="23" t="s">
+      <c r="G30" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="H30" s="14"/>
-    </row>
-    <row r="31" spans="1:8" ht="13.8" customHeight="1">
-      <c r="A31" s="18" t="s">
+      <c r="H30" s="10"/>
+      <c r="J30" s="24"/>
+    </row>
+    <row r="31" spans="1:10" ht="13.8" customHeight="1">
+      <c r="A31" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B31" s="14" t="s">
+      <c r="B31" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="C31" s="22" t="s">
+      <c r="C31" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="D31" s="14" t="s">
+      <c r="D31" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E31" s="19">
+      <c r="E31" s="15">
         <v>98000</v>
       </c>
-      <c r="F31" s="18">
+      <c r="F31" s="14">
         <v>88000</v>
       </c>
-      <c r="G31" s="23" t="s">
+      <c r="G31" s="18" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="32" spans="1:8">
-      <c r="A32" s="14" t="s">
+      <c r="J31" s="24"/>
+    </row>
+    <row r="32" spans="1:10">
+      <c r="A32" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B32" s="14" t="s">
+      <c r="B32" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="22" t="s">
+      <c r="C32" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="D32" s="14" t="s">
+      <c r="D32" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E32" s="19">
+      <c r="E32" s="15">
         <v>150000</v>
       </c>
-      <c r="F32" s="20">
+      <c r="F32" s="16">
         <v>125000</v>
       </c>
-      <c r="G32" s="23" t="s">
+      <c r="G32" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="H32" s="14"/>
-    </row>
-    <row r="33" spans="1:8" ht="17.399999999999999" customHeight="1">
-      <c r="A33" s="14" t="s">
+      <c r="H32" s="10"/>
+      <c r="J32" s="24"/>
+    </row>
+    <row r="33" spans="1:10" ht="17.399999999999999" customHeight="1">
+      <c r="A33" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B33" s="14" t="s">
+      <c r="B33" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C33" s="22" t="s">
+      <c r="C33" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="D33" s="14" t="s">
+      <c r="D33" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E33" s="19">
+      <c r="E33" s="15">
         <v>65000</v>
       </c>
-      <c r="F33" s="20">
+      <c r="F33" s="16">
         <v>62000</v>
       </c>
-      <c r="G33" s="23" t="s">
+      <c r="G33" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="H33" s="14"/>
-    </row>
-    <row r="34" spans="1:8">
-      <c r="A34" s="14" t="s">
+      <c r="H33" s="10"/>
+      <c r="J33" s="25"/>
+    </row>
+    <row r="34" spans="1:10">
+      <c r="A34" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B34" s="14" t="s">
+      <c r="B34" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C34" s="22" t="s">
+      <c r="C34" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="D34" s="14" t="s">
+      <c r="D34" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E34" s="19">
+      <c r="E34" s="15">
         <v>54000</v>
       </c>
-      <c r="F34" s="20">
+      <c r="F34" s="16">
         <v>50000</v>
       </c>
-      <c r="G34" s="23" t="s">
+      <c r="G34" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="H34" s="14"/>
-    </row>
-    <row r="35" spans="1:8" ht="17.399999999999999" customHeight="1">
-      <c r="A35" s="14" t="s">
+      <c r="H34" s="10"/>
+      <c r="J34" s="25"/>
+    </row>
+    <row r="35" spans="1:10" ht="17.399999999999999" customHeight="1">
+      <c r="A35" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B35" s="14" t="s">
+      <c r="B35" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C35" s="22" t="s">
+      <c r="C35" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="D35" s="14" t="s">
+      <c r="D35" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E35" s="19">
+      <c r="E35" s="15">
         <v>96000</v>
       </c>
-      <c r="F35" s="20">
+      <c r="F35" s="16">
         <v>44000</v>
       </c>
-      <c r="G35" s="23" t="s">
+      <c r="G35" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="H35" s="14"/>
-    </row>
-    <row r="36" spans="1:8">
-      <c r="A36" s="14" t="s">
+      <c r="H35" s="10"/>
+      <c r="J35" s="25"/>
+    </row>
+    <row r="36" spans="1:10">
+      <c r="A36" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B36" s="21" t="s">
+      <c r="B36" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="C36" s="22" t="s">
+      <c r="C36" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="D36" s="14" t="s">
+      <c r="D36" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E36" s="19">
+      <c r="E36" s="15">
         <v>50000</v>
       </c>
-      <c r="F36" s="18">
+      <c r="F36" s="14">
         <v>23611</v>
       </c>
-      <c r="G36" s="23" t="s">
+      <c r="G36" s="18" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="37" spans="1:8">
-      <c r="A37" s="14" t="s">
+      <c r="J36" s="25"/>
+    </row>
+    <row r="37" spans="1:10">
+      <c r="A37" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B37" s="21" t="s">
+      <c r="B37" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="C37" s="22" t="s">
+      <c r="C37" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="D37" s="14" t="s">
+      <c r="D37" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E37" s="19">
+      <c r="E37" s="15">
         <v>61500</v>
       </c>
-      <c r="F37" s="18">
+      <c r="F37" s="14">
         <v>22775</v>
       </c>
-      <c r="G37" s="23" t="s">
+      <c r="G37" s="18" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="38" spans="1:8">
-      <c r="A38" s="14" t="s">
+      <c r="J37" s="25"/>
+    </row>
+    <row r="38" spans="1:10">
+      <c r="A38" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B38" s="21" t="s">
+      <c r="B38" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="C38" s="22" t="s">
+      <c r="C38" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="D38" s="14" t="s">
+      <c r="D38" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E38" s="19">
+      <c r="E38" s="15">
         <v>26000</v>
       </c>
-      <c r="F38" s="18">
+      <c r="F38" s="14">
         <v>12600</v>
       </c>
-      <c r="G38" s="23" t="s">
+      <c r="G38" s="18" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="39" spans="1:8">
-      <c r="A39" s="14" t="s">
+      <c r="J38" s="25"/>
+    </row>
+    <row r="39" spans="1:10">
+      <c r="A39" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B39" s="21" t="s">
+      <c r="B39" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C39" s="22" t="s">
+      <c r="C39" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="D39" s="14" t="s">
+      <c r="D39" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E39" s="19">
+      <c r="E39" s="15">
         <v>38000</v>
       </c>
-      <c r="F39" s="18">
+      <c r="F39" s="14">
         <v>37500</v>
       </c>
-      <c r="G39" s="23" t="s">
+      <c r="G39" s="18" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="40" spans="1:8">
-      <c r="A40" s="14" t="s">
+      <c r="J39" s="25"/>
+    </row>
+    <row r="40" spans="1:10">
+      <c r="A40" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B40" s="21" t="s">
+      <c r="B40" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="C40" s="22" t="s">
+      <c r="C40" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="D40" s="14" t="s">
+      <c r="D40" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E40" s="19">
+      <c r="E40" s="15">
         <v>14000</v>
       </c>
-      <c r="F40" s="18">
+      <c r="F40" s="14">
         <v>6396</v>
       </c>
-      <c r="G40" s="23" t="s">
+      <c r="G40" s="18" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="41" spans="1:8">
-      <c r="A41" s="14" t="s">
+      <c r="J40" s="25"/>
+    </row>
+    <row r="41" spans="1:10">
+      <c r="A41" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B41" s="21" t="s">
+      <c r="B41" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="C41" s="22" t="s">
+      <c r="C41" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="D41" s="14" t="s">
+      <c r="D41" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E41" s="19">
+      <c r="E41" s="15">
         <v>12900</v>
       </c>
-      <c r="F41" s="18">
+      <c r="F41" s="14">
         <v>11900</v>
       </c>
-      <c r="G41" s="23" t="s">
+      <c r="G41" s="18" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="42" spans="1:8">
-      <c r="A42" s="14" t="s">
+      <c r="J41" s="25"/>
+    </row>
+    <row r="42" spans="1:10">
+      <c r="A42" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B42" s="21" t="s">
+      <c r="B42" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="C42" s="22" t="s">
+      <c r="C42" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D42" s="14" t="s">
+      <c r="D42" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E42" s="19">
+      <c r="E42" s="15">
         <v>19900</v>
       </c>
-      <c r="F42" s="18">
+      <c r="F42" s="14">
         <v>18900</v>
       </c>
-      <c r="G42" s="23" t="s">
+      <c r="G42" s="18" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="43" spans="1:8">
-      <c r="A43" s="14" t="s">
+      <c r="J42" s="25"/>
+    </row>
+    <row r="43" spans="1:10">
+      <c r="A43" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B43" s="21" t="s">
+      <c r="B43" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="C43" s="22" t="s">
+      <c r="C43" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="D43" s="14" t="s">
+      <c r="D43" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E43" s="19">
+      <c r="E43" s="15">
         <v>22000</v>
       </c>
-      <c r="G43" s="23" t="s">
+      <c r="F43" s="14">
+        <v>1</v>
+      </c>
+      <c r="G43" s="18" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
-      <c r="A44" s="14" t="s">
+    <row r="44" spans="1:10">
+      <c r="A44" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B44" s="21" t="s">
+      <c r="B44" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C44" s="22" t="s">
+      <c r="C44" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="D44" s="14" t="s">
+      <c r="D44" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E44" s="19">
+      <c r="E44" s="15">
         <v>22000</v>
       </c>
-      <c r="G44" s="23" t="s">
+      <c r="F44" s="14">
+        <v>1</v>
+      </c>
+      <c r="G44" s="18" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
-      <c r="A45" s="14" t="s">
+    <row r="45" spans="1:10">
+      <c r="A45" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B45" s="21" t="s">
+      <c r="B45" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="C45" s="22" t="s">
+      <c r="C45" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D45" s="14" t="s">
+      <c r="D45" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E45" s="19">
+      <c r="E45" s="15">
         <v>25200</v>
       </c>
-      <c r="F45" s="18">
+      <c r="F45" s="14">
         <v>12600</v>
       </c>
-      <c r="G45" s="23" t="s">
+      <c r="G45" s="18" t="s">
         <v>154</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="F2:F45">
-    <cfRule type="expression" dxfId="13" priority="1">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>AND($A2="Y",$F2="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J1:J42">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>AND($A1="Y",$F1="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -2503,10 +2573,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="14.4">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="8"/>
+      <c r="B1" s="20"/>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="6" t="s">
@@ -2623,15 +2693,15 @@
       <c r="M1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="O1" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="P1" s="10"/>
-      <c r="Q1" s="10"/>
-      <c r="R1" s="10"/>
-      <c r="S1" s="10"/>
-      <c r="T1" s="10"/>
-      <c r="U1" s="10"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
+      <c r="R1" s="22"/>
+      <c r="S1" s="22"/>
+      <c r="T1" s="22"/>
+      <c r="U1" s="22"/>
     </row>
     <row r="2" spans="1:21">
       <c r="D2" s="3"/>

</xml_diff>

<commit_message>
Update product master unit costs
</commit_message>
<xml_diff>
--- a/유월의보리_product_master.xlsx
+++ b/유월의보리_product_master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\STAND UP\Desktop\HQ\본사 물류마감 자료\26_05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E99D747-4CF7-4D52-A7BF-9A7B4FEE266E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2230E874-A676-464E-A022-3FD2E04EC749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-2100" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PRODUCT_MASTER" sheetId="1" r:id="rId1"/>
@@ -842,6 +842,13 @@
     <xf numFmtId="49" fontId="9" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
+    <xf numFmtId="3" fontId="15" fillId="7" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -852,13 +859,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="15" fillId="7" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -871,6 +871,20 @@
     <cellStyle name="표준 3" xfId="3" xr:uid="{5BFFED80-3383-433D-A609-A987DBFBC66D}"/>
   </cellStyles>
   <dxfs count="15">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <fill>
@@ -897,20 +911,6 @@
           <color indexed="64"/>
         </horizontal>
       </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -1239,7 +1239,7 @@
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="공급단가(ERP)" dataDxfId="5"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="제조원가(입력)" dataDxfId="4"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="팩/단위" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="비고" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="비고" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1454,7 +1454,7 @@
       <c r="H1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="23"/>
+      <c r="J1" s="19"/>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="10" t="s">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="G2" s="10"/>
       <c r="H2" s="10"/>
-      <c r="J2" s="23"/>
+      <c r="J2" s="19"/>
     </row>
     <row r="3" spans="1:10" ht="17.399999999999999">
       <c r="A3" s="10" t="s">
@@ -1498,7 +1498,7 @@
       <c r="F3" s="12">
         <v>28000</v>
       </c>
-      <c r="J3" s="23"/>
+      <c r="J3" s="19"/>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="10" t="s">
@@ -1523,7 +1523,7 @@
         <v>138</v>
       </c>
       <c r="H4" s="10"/>
-      <c r="J4" s="23"/>
+      <c r="J4" s="19"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="10" t="s">
@@ -1548,7 +1548,7 @@
         <v>138</v>
       </c>
       <c r="H5" s="10"/>
-      <c r="J5" s="23"/>
+      <c r="J5" s="19"/>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="10" t="s">
@@ -1573,7 +1573,7 @@
         <v>138</v>
       </c>
       <c r="H6" s="10"/>
-      <c r="J6" s="23"/>
+      <c r="J6" s="19"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="10" t="s">
@@ -1598,7 +1598,7 @@
         <v>138</v>
       </c>
       <c r="H7" s="10"/>
-      <c r="J7" s="23"/>
+      <c r="J7" s="19"/>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="10" t="s">
@@ -1623,7 +1623,7 @@
         <v>138</v>
       </c>
       <c r="H8" s="10"/>
-      <c r="J8" s="23"/>
+      <c r="J8" s="19"/>
     </row>
     <row r="9" spans="1:10" ht="17.399999999999999" customHeight="1">
       <c r="A9" s="10" t="s">
@@ -1648,7 +1648,7 @@
         <v>138</v>
       </c>
       <c r="H9" s="10"/>
-      <c r="J9" s="23"/>
+      <c r="J9" s="19"/>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="10" t="s">
@@ -1673,7 +1673,7 @@
         <v>138</v>
       </c>
       <c r="H10" s="10"/>
-      <c r="J10" s="23"/>
+      <c r="J10" s="19"/>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="10" t="s">
@@ -1698,7 +1698,7 @@
         <v>138</v>
       </c>
       <c r="H11" s="10"/>
-      <c r="J11" s="24"/>
+      <c r="J11" s="20"/>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="10" t="s">
@@ -1723,7 +1723,7 @@
         <v>138</v>
       </c>
       <c r="H12" s="10"/>
-      <c r="J12" s="24"/>
+      <c r="J12" s="20"/>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="10" t="s">
@@ -1748,7 +1748,7 @@
         <v>138</v>
       </c>
       <c r="H13" s="10"/>
-      <c r="J13" s="24"/>
+      <c r="J13" s="20"/>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="10" t="s">
@@ -1773,7 +1773,7 @@
         <v>138</v>
       </c>
       <c r="H14" s="10"/>
-      <c r="J14" s="24"/>
+      <c r="J14" s="20"/>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="10" t="s">
@@ -1798,7 +1798,7 @@
         <v>138</v>
       </c>
       <c r="H15" s="10"/>
-      <c r="J15" s="24"/>
+      <c r="J15" s="20"/>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="10" t="s">
@@ -1823,7 +1823,7 @@
         <v>139</v>
       </c>
       <c r="H16" s="10"/>
-      <c r="J16" s="24"/>
+      <c r="J16" s="20"/>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="10" t="s">
@@ -1848,7 +1848,7 @@
         <v>140</v>
       </c>
       <c r="H17" s="10"/>
-      <c r="J17" s="24"/>
+      <c r="J17" s="20"/>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="10" t="s">
@@ -1873,7 +1873,7 @@
         <v>140</v>
       </c>
       <c r="H18" s="10"/>
-      <c r="J18" s="24"/>
+      <c r="J18" s="20"/>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="10" t="s">
@@ -1898,7 +1898,7 @@
         <v>140</v>
       </c>
       <c r="H19" s="10"/>
-      <c r="J19" s="24"/>
+      <c r="J19" s="20"/>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="10" t="s">
@@ -1923,7 +1923,7 @@
         <v>140</v>
       </c>
       <c r="H20" s="10"/>
-      <c r="J20" s="24"/>
+      <c r="J20" s="20"/>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="10" t="s">
@@ -1948,7 +1948,7 @@
         <v>140</v>
       </c>
       <c r="H21" s="10"/>
-      <c r="J21" s="24"/>
+      <c r="J21" s="20"/>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="10" t="s">
@@ -1973,7 +1973,7 @@
         <v>141</v>
       </c>
       <c r="H22" s="10"/>
-      <c r="J22" s="24"/>
+      <c r="J22" s="20"/>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="10" t="s">
@@ -1998,7 +1998,7 @@
         <v>138</v>
       </c>
       <c r="H23" s="10"/>
-      <c r="J23" s="24"/>
+      <c r="J23" s="20"/>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="10" t="s">
@@ -2023,7 +2023,7 @@
         <v>142</v>
       </c>
       <c r="H24" s="10"/>
-      <c r="J24" s="24"/>
+      <c r="J24" s="20"/>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="10" t="s">
@@ -2048,7 +2048,7 @@
         <v>140</v>
       </c>
       <c r="H25" s="10"/>
-      <c r="J25" s="24"/>
+      <c r="J25" s="20"/>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="10" t="s">
@@ -2073,7 +2073,7 @@
         <v>140</v>
       </c>
       <c r="H26" s="10"/>
-      <c r="J26" s="24"/>
+      <c r="J26" s="20"/>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="10" t="s">
@@ -2098,7 +2098,7 @@
         <v>143</v>
       </c>
       <c r="H27" s="10"/>
-      <c r="J27" s="24"/>
+      <c r="J27" s="20"/>
     </row>
     <row r="28" spans="1:10" ht="17.399999999999999" customHeight="1">
       <c r="A28" s="10" t="s">
@@ -2123,7 +2123,7 @@
         <v>144</v>
       </c>
       <c r="H28" s="10"/>
-      <c r="J28" s="25"/>
+      <c r="J28" s="21"/>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="10" t="s">
@@ -2148,7 +2148,7 @@
         <v>145</v>
       </c>
       <c r="H29" s="10"/>
-      <c r="J29" s="24"/>
+      <c r="J29" s="20"/>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="10" t="s">
@@ -2173,7 +2173,7 @@
         <v>146</v>
       </c>
       <c r="H30" s="10"/>
-      <c r="J30" s="24"/>
+      <c r="J30" s="20"/>
     </row>
     <row r="31" spans="1:10" ht="13.8" customHeight="1">
       <c r="A31" s="14" t="s">
@@ -2197,7 +2197,7 @@
       <c r="G31" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="J31" s="24"/>
+      <c r="J31" s="20"/>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="10" t="s">
@@ -2222,7 +2222,7 @@
         <v>147</v>
       </c>
       <c r="H32" s="10"/>
-      <c r="J32" s="24"/>
+      <c r="J32" s="20"/>
     </row>
     <row r="33" spans="1:10" ht="17.399999999999999" customHeight="1">
       <c r="A33" s="10" t="s">
@@ -2247,7 +2247,7 @@
         <v>148</v>
       </c>
       <c r="H33" s="10"/>
-      <c r="J33" s="25"/>
+      <c r="J33" s="21"/>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="10" t="s">
@@ -2272,7 +2272,7 @@
         <v>149</v>
       </c>
       <c r="H34" s="10"/>
-      <c r="J34" s="25"/>
+      <c r="J34" s="21"/>
     </row>
     <row r="35" spans="1:10" ht="17.399999999999999" customHeight="1">
       <c r="A35" s="10" t="s">
@@ -2291,13 +2291,13 @@
         <v>96000</v>
       </c>
       <c r="F35" s="16">
-        <v>44000</v>
+        <v>88000</v>
       </c>
       <c r="G35" s="18" t="s">
         <v>150</v>
       </c>
       <c r="H35" s="10"/>
-      <c r="J35" s="25"/>
+      <c r="J35" s="21"/>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="10" t="s">
@@ -2321,7 +2321,7 @@
       <c r="G36" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="J36" s="25"/>
+      <c r="J36" s="21"/>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="10" t="s">
@@ -2345,7 +2345,7 @@
       <c r="G37" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="J37" s="25"/>
+      <c r="J37" s="21"/>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="10" t="s">
@@ -2369,7 +2369,7 @@
       <c r="G38" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="J38" s="25"/>
+      <c r="J38" s="21"/>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="10" t="s">
@@ -2393,7 +2393,7 @@
       <c r="G39" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="J39" s="25"/>
+      <c r="J39" s="21"/>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="10" t="s">
@@ -2417,7 +2417,7 @@
       <c r="G40" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="J40" s="25"/>
+      <c r="J40" s="21"/>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="10" t="s">
@@ -2441,7 +2441,7 @@
       <c r="G41" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="J41" s="25"/>
+      <c r="J41" s="21"/>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="10" t="s">
@@ -2465,7 +2465,7 @@
       <c r="G42" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="J42" s="25"/>
+      <c r="J42" s="21"/>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="10" t="s">
@@ -2484,7 +2484,7 @@
         <v>22000</v>
       </c>
       <c r="F43" s="14">
-        <v>1</v>
+        <v>9000</v>
       </c>
       <c r="G43" s="18" t="s">
         <v>140</v>
@@ -2507,7 +2507,7 @@
         <v>22000</v>
       </c>
       <c r="F44" s="14">
-        <v>1</v>
+        <v>9000</v>
       </c>
       <c r="G44" s="18" t="s">
         <v>140</v>
@@ -2539,12 +2539,12 @@
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="F2:F45">
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>AND($A2="Y",$F2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J42">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>AND($A1="Y",$F1="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2573,10 +2573,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="14.4">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="20"/>
+      <c r="B1" s="23"/>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="6" t="s">
@@ -2693,15 +2693,15 @@
       <c r="M1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="O1" s="21" t="s">
+      <c r="O1" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="22"/>
-      <c r="T1" s="22"/>
-      <c r="U1" s="22"/>
+      <c r="P1" s="25"/>
+      <c r="Q1" s="25"/>
+      <c r="R1" s="25"/>
+      <c r="S1" s="25"/>
+      <c r="T1" s="25"/>
+      <c r="U1" s="25"/>
     </row>
     <row r="2" spans="1:21">
       <c r="D2" s="3"/>

</xml_diff>